<commit_message>
Changing item upgrade cost
</commit_message>
<xml_diff>
--- a/Calculations.xlsx
+++ b/Calculations.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14685" windowHeight="12720" firstSheet="3" activeTab="9"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14690" windowHeight="12720" firstSheet="3" activeTab="11"/>
   </bookViews>
   <sheets>
     <sheet name="Creatures Per Level" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="93">
   <si>
     <t>Width</t>
   </si>
@@ -312,6 +312,9 @@
   <si>
     <t>Prob</t>
   </si>
+  <si>
+    <t>Power</t>
+  </si>
 </sst>
 </file>
 
@@ -498,7 +501,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
@@ -572,6 +575,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1033,11 +1037,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="266602880"/>
-        <c:axId val="266601312"/>
+        <c:axId val="247560272"/>
+        <c:axId val="247559096"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="266602880"/>
+        <c:axId val="247560272"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="200"/>
@@ -1095,12 +1099,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="266601312"/>
+        <c:crossAx val="247559096"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="266601312"/>
+        <c:axId val="247559096"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -1158,7 +1162,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="266602880"/>
+        <c:crossAx val="247560272"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1963,11 +1967,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="266612288"/>
-        <c:axId val="266610720"/>
+        <c:axId val="247559488"/>
+        <c:axId val="320460992"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="266612288"/>
+        <c:axId val="247559488"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="60"/>
@@ -2025,12 +2029,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="266610720"/>
+        <c:crossAx val="320460992"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="266610720"/>
+        <c:axId val="320460992"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2087,7 +2091,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="266612288"/>
+        <c:crossAx val="247559488"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2151,6 +2155,31 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Success Probability</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
@@ -2227,144 +2256,376 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Build Diff'!$B$3:$B$23</c:f>
+              <c:f>'Build Diff'!$B$3:$B$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="21"/>
+                <c:ptCount val="25"/>
                 <c:pt idx="0">
+                  <c:v>-12</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-11</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>-10</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="3">
                   <c:v>-9</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="4">
                   <c:v>-8</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="5">
                   <c:v>-7</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="6">
                   <c:v>-6</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="7">
                   <c:v>-5</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="8">
                   <c:v>-4</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="9">
                   <c:v>-3</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="10">
                   <c:v>-2</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="11">
                   <c:v>-1</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="12">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="13">
                   <c:v>1</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="14">
                   <c:v>2</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="15">
                   <c:v>3</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="16">
                   <c:v>4</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="17">
                   <c:v>5</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="18">
                   <c:v>6</c:v>
                 </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="19">
                   <c:v>7</c:v>
                 </c:pt>
-                <c:pt idx="18">
+                <c:pt idx="20">
                   <c:v>8</c:v>
                 </c:pt>
-                <c:pt idx="19">
+                <c:pt idx="21">
                   <c:v>9</c:v>
                 </c:pt>
-                <c:pt idx="20">
+                <c:pt idx="22">
                   <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>12</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Build Diff'!$C$3:$C$23</c:f>
+              <c:f>'Build Diff'!$C$3:$C$27</c:f>
+              <c:numCache>
+                <c:formatCode>0.00%</c:formatCode>
+                <c:ptCount val="25"/>
+                <c:pt idx="0">
+                  <c:v>2.2820382366630199E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3.1266634947545169E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4.2834554246828152E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5.867006903530491E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8.0326076718705883E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.10988306244092602</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.15006332390515698</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.20425466859955624</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.2762180271064601</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.36899071958615975</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.48230053894349789</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.60869757828200788</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.73204284797281272</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.8340735241978966</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.90557259430520598</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.94934425992620519</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.97378496795878799</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.98670152829719915</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.9933244664310189</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.9966670193856727</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.99834040910438182</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.99917476132312211</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.99958992419987602</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.99979629464133524</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.99989882619802406</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Build Diff'!$D$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Current</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Build Diff'!$B$3:$B$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="21"/>
+                <c:ptCount val="25"/>
                 <c:pt idx="0">
-                  <c:v>1.8312567555274113E-2</c:v>
+                  <c:v>-12</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.7313528403278421E-2</c:v>
+                  <c:v>-11</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.0728381752463738E-2</c:v>
+                  <c:v>-10</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>6.0697939828597031E-2</c:v>
+                  <c:v>-9</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>9.0346948776147878E-2</c:v>
+                  <c:v>-8</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.13411267636614951</c:v>
+                  <c:v>-7</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.1979033167907106</c:v>
+                  <c:v>-6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.28839676921547225</c:v>
+                  <c:v>-5</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.40985560245783575</c:v>
+                  <c:v>-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.55679935243531631</c:v>
+                  <c:v>-3</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.70710678118654757</c:v>
+                  <c:v>-2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.83064702559367087</c:v>
+                  <c:v>-1</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.91215041804185149</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.95751099393483607</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.9802215449597278</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.99096608924720953</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.99591035181227039</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.99815618021458152</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.99917025522171421</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.9996269159872414</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.99983231087494551</c:v>
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>12</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Build Diff'!$D$3:$D$27</c:f>
+              <c:numCache>
+                <c:formatCode>0.00%</c:formatCode>
+                <c:ptCount val="25"/>
+                <c:pt idx="0">
+                  <c:v>6.1701267704311075E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>9.4279190270153083E-3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.4405030899737827E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.2006981328636856E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3.3611739116658539E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5.1305554746093711E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7.8211082956288397E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.11888252458819391</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.17957267711276778</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.26766390785711713</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.3884979473670771</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.53757695724874877</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.69255473405546231</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.82145070207510695</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.90713192022269118</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.95501984306226939</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.9790473552534269</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.9904266572276561</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.9956655054659711</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.99804565919952104</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.99912049243426082</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.99960453537328886</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.99982225042169381</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.99992012068103908</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.9999641056294265</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2379,15 +2640,15 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="266602096"/>
-        <c:axId val="266602488"/>
+        <c:axId val="320461384"/>
+        <c:axId val="320463344"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="266602096"/>
+        <c:axId val="320461384"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="10"/>
-          <c:min val="-10"/>
+          <c:max val="12"/>
+          <c:min val="-12"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -2442,12 +2703,13 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="266602488"/>
+        <c:crossAx val="320463344"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
+        <c:majorUnit val="4"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="266602488"/>
+        <c:axId val="320463344"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -2468,7 +2730,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00%" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2505,7 +2767,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="266602096"/>
+        <c:crossAx val="320461384"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4296,13 +4558,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>28575</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>166687</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>428625</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
@@ -4591,13 +4853,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B4:M34"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="5" max="6" width="10.5703125" customWidth="1"/>
-    <col min="12" max="12" width="11.42578125" customWidth="1"/>
+    <col min="5" max="6" width="10.54296875" customWidth="1"/>
+    <col min="12" max="12" width="11.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B4" s="8" t="s">
         <v>0</v>
       </c>
@@ -4629,7 +4891,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B5">
         <v>20</v>
       </c>
@@ -4665,7 +4927,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B6">
         <v>20</v>
       </c>
@@ -4695,7 +4957,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B7">
         <v>20</v>
       </c>
@@ -4725,7 +4987,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B8">
         <v>30</v>
       </c>
@@ -4755,7 +5017,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B9">
         <v>30</v>
       </c>
@@ -4785,7 +5047,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B10">
         <v>30</v>
       </c>
@@ -4815,7 +5077,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B11">
         <v>30</v>
       </c>
@@ -4845,7 +5107,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B12">
         <v>30</v>
       </c>
@@ -4878,7 +5140,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B13">
         <v>30</v>
       </c>
@@ -4908,7 +5170,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B14">
         <v>35</v>
       </c>
@@ -4938,7 +5200,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B15">
         <v>35</v>
       </c>
@@ -4968,7 +5230,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B16">
         <v>40</v>
       </c>
@@ -4998,7 +5260,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B17">
         <v>40</v>
       </c>
@@ -5028,7 +5290,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B18">
         <v>50</v>
       </c>
@@ -5058,7 +5320,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B19">
         <v>50</v>
       </c>
@@ -5088,7 +5350,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B20">
         <v>20</v>
       </c>
@@ -5118,7 +5380,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B21">
         <v>20</v>
       </c>
@@ -5148,7 +5410,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B22">
         <v>20</v>
       </c>
@@ -5178,7 +5440,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B23">
         <v>30</v>
       </c>
@@ -5208,7 +5470,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B24">
         <v>30</v>
       </c>
@@ -5238,7 +5500,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B25">
         <v>30</v>
       </c>
@@ -5268,7 +5530,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B26">
         <v>30</v>
       </c>
@@ -5298,7 +5560,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B27">
         <v>30</v>
       </c>
@@ -5328,7 +5590,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B28">
         <v>30</v>
       </c>
@@ -5358,7 +5620,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B29">
         <v>35</v>
       </c>
@@ -5388,7 +5650,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B30">
         <v>35</v>
       </c>
@@ -5418,7 +5680,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B31">
         <v>40</v>
       </c>
@@ -5448,7 +5710,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B32">
         <v>40</v>
       </c>
@@ -5478,7 +5740,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B33">
         <v>50</v>
       </c>
@@ -5508,7 +5770,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B34">
         <v>50</v>
       </c>
@@ -5547,9 +5809,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A2:L53"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="12" t="s">
         <v>20</v>
       </c>
@@ -5578,7 +5840,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>0</v>
       </c>
@@ -5615,7 +5877,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>0.5</v>
       </c>
@@ -5652,7 +5914,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1</v>
       </c>
@@ -5679,7 +5941,7 @@
       <c r="J5" s="13"/>
       <c r="K5" s="13"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1.5</v>
       </c>
@@ -5711,7 +5973,7 @@
       </c>
       <c r="K6" s="13"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>2</v>
       </c>
@@ -5736,7 +5998,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2.5</v>
       </c>
@@ -5761,7 +6023,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>3</v>
       </c>
@@ -5786,7 +6048,7 @@
         <v>3.4</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>3.5</v>
       </c>
@@ -5811,7 +6073,7 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>4</v>
       </c>
@@ -5836,7 +6098,7 @@
         <v>4.2</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>4.5</v>
       </c>
@@ -5861,7 +6123,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>5</v>
       </c>
@@ -5886,7 +6148,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>6</v>
       </c>
@@ -5911,7 +6173,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>7</v>
       </c>
@@ -5936,7 +6198,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>8</v>
       </c>
@@ -5961,7 +6223,7 @@
         <v>5.9</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>9</v>
       </c>
@@ -5986,7 +6248,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>10</v>
       </c>
@@ -6011,7 +6273,7 @@
         <v>6.4</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>11</v>
       </c>
@@ -6036,7 +6298,7 @@
         <v>6.7</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>12</v>
       </c>
@@ -6061,7 +6323,7 @@
         <v>6.9</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>13</v>
       </c>
@@ -6086,7 +6348,7 @@
         <v>7.1</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>14</v>
       </c>
@@ -6111,7 +6373,7 @@
         <v>7.3</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>15</v>
       </c>
@@ -6136,7 +6398,7 @@
         <v>7.6</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>16</v>
       </c>
@@ -6161,7 +6423,7 @@
         <v>7.8</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>17</v>
       </c>
@@ -6186,7 +6448,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>18</v>
       </c>
@@ -6211,7 +6473,7 @@
         <v>8.1999999999999993</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>19</v>
       </c>
@@ -6236,7 +6498,7 @@
         <v>8.4</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>20</v>
       </c>
@@ -6261,7 +6523,7 @@
         <v>8.6</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>21</v>
       </c>
@@ -6286,7 +6548,7 @@
         <v>8.8000000000000007</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>22</v>
       </c>
@@ -6311,7 +6573,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>23</v>
       </c>
@@ -6336,7 +6598,7 @@
         <v>9.1999999999999993</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>24</v>
       </c>
@@ -6361,7 +6623,7 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>25</v>
       </c>
@@ -6386,7 +6648,7 @@
         <v>9.6</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>26</v>
       </c>
@@ -6411,7 +6673,7 @@
         <v>9.8000000000000007</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>27</v>
       </c>
@@ -6436,7 +6698,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>28</v>
       </c>
@@ -6461,7 +6723,7 @@
         <v>10.199999999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>29</v>
       </c>
@@ -6486,7 +6748,7 @@
         <v>10.4</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>30</v>
       </c>
@@ -6511,7 +6773,7 @@
         <v>10.6</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>32</v>
       </c>
@@ -6536,7 +6798,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>34</v>
       </c>
@@ -6561,7 +6823,7 @@
         <v>11.3</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>36</v>
       </c>
@@ -6586,7 +6848,7 @@
         <v>11.7</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>38</v>
       </c>
@@ -6611,7 +6873,7 @@
         <v>12.1</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>40</v>
       </c>
@@ -6636,7 +6898,7 @@
         <v>12.4</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>42</v>
       </c>
@@ -6661,7 +6923,7 @@
         <v>12.8</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>44</v>
       </c>
@@ -6686,7 +6948,7 @@
         <v>13.2</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>46</v>
       </c>
@@ -6711,7 +6973,7 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>48</v>
       </c>
@@ -6736,7 +6998,7 @@
         <v>13.9</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>50</v>
       </c>
@@ -6761,7 +7023,7 @@
         <v>14.2</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>52</v>
       </c>
@@ -6786,7 +7048,7 @@
         <v>14.6</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>54</v>
       </c>
@@ -6811,7 +7073,7 @@
         <v>14.9</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>56</v>
       </c>
@@ -6836,7 +7098,7 @@
         <v>15.2</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>58</v>
       </c>
@@ -6861,7 +7123,7 @@
         <v>15.6</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>60</v>
       </c>
@@ -6896,14 +7158,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:R41"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B2" s="23" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:18" x14ac:dyDescent="0.35">
       <c r="E3" s="11" t="s">
         <v>35</v>
       </c>
@@ -6914,7 +7176,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="4" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B4" s="18" t="s">
         <v>36</v>
       </c>
@@ -6947,7 +7209,7 @@
       <c r="Q4" s="24"/>
       <c r="R4" s="24"/>
     </row>
-    <row r="5" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B5" s="21">
         <v>0</v>
       </c>
@@ -6985,7 +7247,7 @@
       <c r="Q5" s="24"/>
       <c r="R5" s="24"/>
     </row>
-    <row r="6" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B6" s="21">
         <v>10</v>
       </c>
@@ -7021,7 +7283,7 @@
       <c r="Q6" s="24"/>
       <c r="R6" s="24"/>
     </row>
-    <row r="7" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B7" s="21">
         <v>20</v>
       </c>
@@ -7059,7 +7321,7 @@
       <c r="Q7" s="24"/>
       <c r="R7" s="24"/>
     </row>
-    <row r="8" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B8" s="21">
         <v>30</v>
       </c>
@@ -7097,7 +7359,7 @@
       <c r="Q8" s="24"/>
       <c r="R8" s="24"/>
     </row>
-    <row r="9" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B9" s="21">
         <v>40</v>
       </c>
@@ -7129,7 +7391,7 @@
       <c r="Q9" s="24"/>
       <c r="R9" s="24"/>
     </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B10" s="21">
         <v>50</v>
       </c>
@@ -7161,7 +7423,7 @@
       <c r="Q10" s="24"/>
       <c r="R10" s="24"/>
     </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B11" s="21">
         <v>60</v>
       </c>
@@ -7186,7 +7448,7 @@
         <v>120.4241430025403</v>
       </c>
     </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B12" s="21">
         <v>70</v>
       </c>
@@ -7211,7 +7473,7 @@
         <v>153.76958819994368</v>
       </c>
     </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B13" s="21">
         <v>80</v>
       </c>
@@ -7236,7 +7498,7 @@
         <v>196.34838717250804</v>
       </c>
     </row>
-    <row r="14" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B14" s="21">
         <v>90</v>
       </c>
@@ -7261,7 +7523,7 @@
         <v>250.71725558057545</v>
       </c>
     </row>
-    <row r="15" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B15" s="21">
         <v>100</v>
       </c>
@@ -7286,7 +7548,7 @@
         <v>320.14086365083676</v>
       </c>
     </row>
-    <row r="16" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B16" s="21">
         <v>110</v>
       </c>
@@ -7311,7 +7573,7 @@
         <v>408.78786879575335</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B17" s="21">
         <v>120</v>
       </c>
@@ -7336,7 +7598,7 @@
         <v>521.98122966529729</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B18" s="21">
         <v>130</v>
       </c>
@@ -7361,7 +7623,7 @@
         <v>666.51783215961791</v>
       </c>
     </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B19" s="21">
         <v>140</v>
       </c>
@@ -7386,17 +7648,17 @@
         <v>851.07661988461609</v>
       </c>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B24" s="23" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.35">
       <c r="E25" s="11" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B26" s="18" t="s">
         <v>36</v>
       </c>
@@ -7416,7 +7678,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B27" s="21">
         <v>0</v>
       </c>
@@ -7441,7 +7703,7 @@
         <v>63.418220571798358</v>
       </c>
     </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B28" s="21">
         <v>10</v>
       </c>
@@ -7466,7 +7728,7 @@
         <v>63.418220571798358</v>
       </c>
     </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B29" s="21">
         <v>20</v>
       </c>
@@ -7491,7 +7753,7 @@
         <v>63.418220571798358</v>
       </c>
     </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B30" s="21">
         <v>30</v>
       </c>
@@ -7516,7 +7778,7 @@
         <v>80.978725848129301</v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B31" s="21">
         <v>40</v>
       </c>
@@ -7541,7 +7803,7 @@
         <v>103.40173503547628</v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B32" s="21">
         <v>50</v>
       </c>
@@ -7566,7 +7828,7 @@
         <v>132.03367546679962</v>
       </c>
     </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B33" s="21">
         <v>60</v>
       </c>
@@ -7591,7 +7853,7 @@
         <v>168.59380020355641</v>
       </c>
     </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B34" s="21">
         <v>70</v>
       </c>
@@ -7616,7 +7878,7 @@
         <v>215.27742347992114</v>
       </c>
     </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B35" s="21">
         <v>80</v>
       </c>
@@ -7641,7 +7903,7 @@
         <v>274.88774204151122</v>
       </c>
     </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B36" s="21">
         <v>90</v>
       </c>
@@ -7666,7 +7928,7 @@
         <v>351.00415781280554</v>
       </c>
     </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B37" s="21">
         <v>100</v>
       </c>
@@ -7691,7 +7953,7 @@
         <v>448.19720911117139</v>
       </c>
     </row>
-    <row r="38" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B38" s="21">
         <v>110</v>
       </c>
@@ -7716,7 +7978,7 @@
         <v>572.30301631405462</v>
       </c>
     </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B39" s="21">
         <v>120</v>
       </c>
@@ -7741,7 +8003,7 @@
         <v>730.77372153141607</v>
       </c>
     </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B40" s="21">
         <v>130</v>
       </c>
@@ -7766,7 +8028,7 @@
         <v>933.12496502346505</v>
       </c>
     </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B41" s="21">
         <v>140</v>
       </c>
@@ -7799,213 +8061,358 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:F23"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:G27"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="3" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B2" s="12" t="s">
         <v>90</v>
       </c>
       <c r="C2" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="E2" s="40" t="s">
+      <c r="D2" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="F2" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="40">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="40">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B3">
+        <v>-12</v>
+      </c>
+      <c r="C3" s="41">
+        <f>POWER(1/(1+EXP(-$B3*$G$2)), $G$3)</f>
+        <v>2.2820382366630199E-2</v>
+      </c>
+      <c r="D3" s="41">
+        <f>POWER(1/(1+EXP(-$B3*0.8)),0.53)</f>
+        <v>6.1701267704311075E-3</v>
+      </c>
+      <c r="F3" s="40" t="s">
+        <v>92</v>
+      </c>
+      <c r="G3" s="40">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B4">
+        <v>-11</v>
+      </c>
+      <c r="C4" s="41">
+        <f>POWER(1/(1+EXP(-$B4*$G$2)), $G$3)</f>
+        <v>3.1266634947545169E-2</v>
+      </c>
+      <c r="D4" s="41">
+        <f>POWER(1/(1+EXP(-$B4*0.8)),0.53)</f>
+        <v>9.4279190270153083E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B5">
         <v>-10</v>
       </c>
-      <c r="C3">
-        <f>SQRT(1/(1+EXP(-$B3*$F$2)))</f>
-        <v>1.8312567555274113E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4">
+      <c r="C5" s="41">
+        <f>POWER(1/(1+EXP(-$B5*$G$2)), $G$3)</f>
+        <v>4.2834554246828152E-2</v>
+      </c>
+      <c r="D5" s="41">
+        <f>POWER(1/(1+EXP(-$B5*0.8)),0.53)</f>
+        <v>1.4405030899737827E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B6">
         <v>-9</v>
       </c>
-      <c r="C4">
-        <f t="shared" ref="C4:C23" si="0">SQRT(1/(1+EXP(-$B4*$F$2)))</f>
-        <v>2.7313528403278421E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5">
+      <c r="C6" s="41">
+        <f>POWER(1/(1+EXP(-$B6*$G$2)), $G$3)</f>
+        <v>5.867006903530491E-2</v>
+      </c>
+      <c r="D6" s="41">
+        <f>POWER(1/(1+EXP(-$B6*0.8)),0.53)</f>
+        <v>2.2006981328636856E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B7">
         <v>-8</v>
       </c>
-      <c r="C5">
-        <f t="shared" si="0"/>
-        <v>4.0728381752463738E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6">
+      <c r="C7" s="41">
+        <f>POWER(1/(1+EXP(-$B7*$G$2)), $G$3)</f>
+        <v>8.0326076718705883E-2</v>
+      </c>
+      <c r="D7" s="41">
+        <f>POWER(1/(1+EXP(-$B7*0.8)),0.53)</f>
+        <v>3.3611739116658539E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B8">
         <v>-7</v>
       </c>
-      <c r="C6">
-        <f t="shared" si="0"/>
-        <v>6.0697939828597031E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7">
+      <c r="C8" s="41">
+        <f>POWER(1/(1+EXP(-$B8*$G$2)), $G$3)</f>
+        <v>0.10988306244092602</v>
+      </c>
+      <c r="D8" s="41">
+        <f>POWER(1/(1+EXP(-$B8*0.8)),0.53)</f>
+        <v>5.1305554746093711E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B9">
         <v>-6</v>
       </c>
-      <c r="C7">
-        <f t="shared" si="0"/>
-        <v>9.0346948776147878E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8">
+      <c r="C9" s="41">
+        <f>POWER(1/(1+EXP(-$B9*$G$2)), $G$3)</f>
+        <v>0.15006332390515698</v>
+      </c>
+      <c r="D9" s="41">
+        <f>POWER(1/(1+EXP(-$B9*0.8)),0.53)</f>
+        <v>7.8211082956288397E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B10">
         <v>-5</v>
       </c>
-      <c r="C8">
-        <f t="shared" si="0"/>
-        <v>0.13411267636614951</v>
-      </c>
-    </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9">
+      <c r="C10" s="41">
+        <f>POWER(1/(1+EXP(-$B10*$G$2)), $G$3)</f>
+        <v>0.20425466859955624</v>
+      </c>
+      <c r="D10" s="41">
+        <f>POWER(1/(1+EXP(-$B10*0.8)),0.53)</f>
+        <v>0.11888252458819391</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B11">
         <v>-4</v>
       </c>
-      <c r="C9">
-        <f t="shared" si="0"/>
-        <v>0.1979033167907106</v>
-      </c>
-    </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B10">
+      <c r="C11" s="41">
+        <f>POWER(1/(1+EXP(-$B11*$G$2)), $G$3)</f>
+        <v>0.2762180271064601</v>
+      </c>
+      <c r="D11" s="41">
+        <f>POWER(1/(1+EXP(-$B11*0.8)),0.53)</f>
+        <v>0.17957267711276778</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B12">
         <v>-3</v>
       </c>
-      <c r="C10">
-        <f t="shared" si="0"/>
-        <v>0.28839676921547225</v>
-      </c>
-    </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11">
+      <c r="C12" s="41">
+        <f>POWER(1/(1+EXP(-$B12*$G$2)), $G$3)</f>
+        <v>0.36899071958615975</v>
+      </c>
+      <c r="D12" s="41">
+        <f>POWER(1/(1+EXP(-$B12*0.8)),0.53)</f>
+        <v>0.26766390785711713</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B13">
         <v>-2</v>
       </c>
-      <c r="C11">
-        <f t="shared" si="0"/>
-        <v>0.40985560245783575</v>
-      </c>
-    </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B12">
+      <c r="C13" s="41">
+        <f>POWER(1/(1+EXP(-$B13*$G$2)), $G$3)</f>
+        <v>0.48230053894349789</v>
+      </c>
+      <c r="D13" s="41">
+        <f>POWER(1/(1+EXP(-$B13*0.8)),0.53)</f>
+        <v>0.3884979473670771</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B14">
         <v>-1</v>
       </c>
-      <c r="C12">
-        <f t="shared" si="0"/>
-        <v>0.55679935243531631</v>
-      </c>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13">
+      <c r="C14" s="41">
+        <f>POWER(1/(1+EXP(-$B14*$G$2)), $G$3)</f>
+        <v>0.60869757828200788</v>
+      </c>
+      <c r="D14" s="41">
+        <f>POWER(1/(1+EXP(-$B14*0.8)),0.53)</f>
+        <v>0.53757695724874877</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B15">
         <v>0</v>
       </c>
-      <c r="C13">
-        <f t="shared" si="0"/>
-        <v>0.70710678118654757</v>
-      </c>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14">
+      <c r="C15" s="41">
+        <f>POWER(1/(1+EXP(-$B15*$G$2)), $G$3)</f>
+        <v>0.73204284797281272</v>
+      </c>
+      <c r="D15" s="41">
+        <f>POWER(1/(1+EXP(-$B15*0.8)),0.53)</f>
+        <v>0.69255473405546231</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B16">
         <v>1</v>
       </c>
-      <c r="C14">
-        <f t="shared" si="0"/>
-        <v>0.83064702559367087</v>
-      </c>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B15">
+      <c r="C16" s="41">
+        <f>POWER(1/(1+EXP(-$B16*$G$2)), $G$3)</f>
+        <v>0.8340735241978966</v>
+      </c>
+      <c r="D16" s="41">
+        <f>POWER(1/(1+EXP(-$B16*0.8)),0.53)</f>
+        <v>0.82145070207510695</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B17">
         <v>2</v>
       </c>
-      <c r="C15">
-        <f t="shared" si="0"/>
-        <v>0.91215041804185149</v>
-      </c>
-    </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B16">
+      <c r="C17" s="41">
+        <f>POWER(1/(1+EXP(-$B17*$G$2)), $G$3)</f>
+        <v>0.90557259430520598</v>
+      </c>
+      <c r="D17" s="41">
+        <f>POWER(1/(1+EXP(-$B17*0.8)),0.53)</f>
+        <v>0.90713192022269118</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B18">
         <v>3</v>
       </c>
-      <c r="C16">
-        <f t="shared" si="0"/>
-        <v>0.95751099393483607</v>
-      </c>
-    </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B17">
+      <c r="C18" s="41">
+        <f>POWER(1/(1+EXP(-$B18*$G$2)), $G$3)</f>
+        <v>0.94934425992620519</v>
+      </c>
+      <c r="D18" s="41">
+        <f>POWER(1/(1+EXP(-$B18*0.8)),0.53)</f>
+        <v>0.95501984306226939</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B19">
         <v>4</v>
       </c>
-      <c r="C17">
-        <f t="shared" si="0"/>
-        <v>0.9802215449597278</v>
-      </c>
-    </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B18">
+      <c r="C19" s="41">
+        <f>POWER(1/(1+EXP(-$B19*$G$2)), $G$3)</f>
+        <v>0.97378496795878799</v>
+      </c>
+      <c r="D19" s="41">
+        <f>POWER(1/(1+EXP(-$B19*0.8)),0.53)</f>
+        <v>0.9790473552534269</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B20">
         <v>5</v>
       </c>
-      <c r="C18">
-        <f t="shared" si="0"/>
-        <v>0.99096608924720953</v>
-      </c>
-    </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B19">
+      <c r="C20" s="41">
+        <f>POWER(1/(1+EXP(-$B20*$G$2)), $G$3)</f>
+        <v>0.98670152829719915</v>
+      </c>
+      <c r="D20" s="41">
+        <f>POWER(1/(1+EXP(-$B20*0.8)),0.53)</f>
+        <v>0.9904266572276561</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B21">
         <v>6</v>
       </c>
-      <c r="C19">
-        <f t="shared" si="0"/>
-        <v>0.99591035181227039</v>
-      </c>
-    </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B20">
+      <c r="C21" s="41">
+        <f>POWER(1/(1+EXP(-$B21*$G$2)), $G$3)</f>
+        <v>0.9933244664310189</v>
+      </c>
+      <c r="D21" s="41">
+        <f>POWER(1/(1+EXP(-$B21*0.8)),0.53)</f>
+        <v>0.9956655054659711</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B22">
         <v>7</v>
       </c>
-      <c r="C20">
-        <f t="shared" si="0"/>
-        <v>0.99815618021458152</v>
-      </c>
-    </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B21">
+      <c r="C22" s="41">
+        <f>POWER(1/(1+EXP(-$B22*$G$2)), $G$3)</f>
+        <v>0.9966670193856727</v>
+      </c>
+      <c r="D22" s="41">
+        <f>POWER(1/(1+EXP(-$B22*0.8)),0.53)</f>
+        <v>0.99804565919952104</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B23">
         <v>8</v>
       </c>
-      <c r="C21">
-        <f t="shared" si="0"/>
-        <v>0.99917025522171421</v>
-      </c>
-    </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B22">
+      <c r="C23" s="41">
+        <f>POWER(1/(1+EXP(-$B23*$G$2)), $G$3)</f>
+        <v>0.99834040910438182</v>
+      </c>
+      <c r="D23" s="41">
+        <f>POWER(1/(1+EXP(-$B23*0.8)),0.53)</f>
+        <v>0.99912049243426082</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B24">
         <v>9</v>
       </c>
-      <c r="C22">
-        <f t="shared" si="0"/>
-        <v>0.9996269159872414</v>
-      </c>
-    </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B23">
+      <c r="C24" s="41">
+        <f>POWER(1/(1+EXP(-$B24*$G$2)), $G$3)</f>
+        <v>0.99917476132312211</v>
+      </c>
+      <c r="D24" s="41">
+        <f>POWER(1/(1+EXP(-$B24*0.8)),0.53)</f>
+        <v>0.99960453537328886</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B25">
         <v>10</v>
       </c>
-      <c r="C23">
-        <f t="shared" si="0"/>
-        <v>0.99983231087494551</v>
+      <c r="C25" s="41">
+        <f>POWER(1/(1+EXP(-$B25*$G$2)), $G$3)</f>
+        <v>0.99958992419987602</v>
+      </c>
+      <c r="D25" s="41">
+        <f>POWER(1/(1+EXP(-$B25*0.8)),0.53)</f>
+        <v>0.99982225042169381</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B26">
+        <v>11</v>
+      </c>
+      <c r="C26" s="41">
+        <f>POWER(1/(1+EXP(-$B26*$G$2)), $G$3)</f>
+        <v>0.99979629464133524</v>
+      </c>
+      <c r="D26" s="41">
+        <f>POWER(1/(1+EXP(-$B26*0.8)),0.53)</f>
+        <v>0.99992012068103908</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B27">
+        <v>12</v>
+      </c>
+      <c r="C27" s="41">
+        <f>POWER(1/(1+EXP(-$B27*$G$2)), $G$3)</f>
+        <v>0.99989882619802406</v>
+      </c>
+      <c r="D27" s="41">
+        <f>POWER(1/(1+EXP(-$B27*0.8)),0.53)</f>
+        <v>0.9999641056294265</v>
       </c>
     </row>
   </sheetData>
@@ -8018,16 +8425,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:J22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="6"/>
-    <col min="6" max="6" width="22.28515625" style="16" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.140625" style="17"/>
+    <col min="2" max="2" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.1796875" style="6"/>
+    <col min="6" max="6" width="22.26953125" style="16" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.1796875" style="17"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B2" s="34" t="s">
         <v>4</v>
       </c>
@@ -8044,7 +8451,7 @@
         <v>1.6</v>
       </c>
     </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B3" s="38">
         <v>1</v>
       </c>
@@ -8061,7 +8468,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B4" s="38">
         <v>2</v>
       </c>
@@ -8080,7 +8487,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B5" s="38">
         <v>3</v>
       </c>
@@ -8093,7 +8500,7 @@
         <v>3400</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B6" s="38">
         <v>4</v>
       </c>
@@ -8107,7 +8514,7 @@
       </c>
       <c r="J6" s="19"/>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B7" s="38">
         <v>5</v>
       </c>
@@ -8120,7 +8527,7 @@
         <v>13400</v>
       </c>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B8" s="38">
         <v>6</v>
       </c>
@@ -8133,7 +8540,7 @@
         <v>23200</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B9" s="38">
         <v>7</v>
       </c>
@@ -8146,7 +8553,7 @@
         <v>38900</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B10" s="38">
         <v>8</v>
       </c>
@@ -8159,7 +8566,7 @@
         <v>64100</v>
       </c>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B11" s="38">
         <v>9</v>
       </c>
@@ -8172,7 +8579,7 @@
         <v>104000</v>
       </c>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B12" s="38">
         <v>10</v>
       </c>
@@ -8185,7 +8592,7 @@
         <v>169000</v>
       </c>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B13" s="38">
         <v>11</v>
       </c>
@@ -8198,7 +8605,7 @@
         <v>272000</v>
       </c>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B14" s="38">
         <v>12</v>
       </c>
@@ -8211,7 +8618,7 @@
         <v>437000</v>
       </c>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B15" s="38">
         <v>13</v>
       </c>
@@ -8224,7 +8631,7 @@
         <v>701000</v>
       </c>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B16" s="38">
         <v>14</v>
       </c>
@@ -8237,7 +8644,7 @@
         <v>1120000</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B17" s="38">
         <v>15</v>
       </c>
@@ -8250,7 +8657,7 @@
         <v>1800000</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B18" s="38">
         <v>16</v>
       </c>
@@ -8263,7 +8670,7 @@
         <v>2880000</v>
       </c>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B19" s="38">
         <v>17</v>
       </c>
@@ -8276,7 +8683,7 @@
         <v>4610000</v>
       </c>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B20" s="38">
         <v>18</v>
       </c>
@@ -8289,7 +8696,7 @@
         <v>7380000</v>
       </c>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B21" s="38">
         <v>19</v>
       </c>
@@ -8302,7 +8709,7 @@
         <v>11800000</v>
       </c>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B22" s="38">
         <v>20</v>
       </c>
@@ -8324,13 +8731,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B3:J28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="12.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B3" s="37" t="s">
         <v>4</v>
       </c>
@@ -8350,7 +8757,7 @@
         <v>1.34</v>
       </c>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B4">
         <v>1</v>
       </c>
@@ -8365,7 +8772,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B5">
         <v>2</v>
       </c>
@@ -8380,7 +8787,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B6">
         <v>3</v>
       </c>
@@ -8395,7 +8802,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B7">
         <v>4</v>
       </c>
@@ -8410,7 +8817,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B8">
         <v>5</v>
       </c>
@@ -8425,7 +8832,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B9">
         <v>6</v>
       </c>
@@ -8434,7 +8841,7 @@
         <v>20.262677605856013</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B10">
         <v>7</v>
       </c>
@@ -8443,7 +8850,7 @@
         <v>27.151987991847054</v>
       </c>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B11">
         <v>8</v>
       </c>
@@ -8452,7 +8859,7 @@
         <v>36.383663909075061</v>
       </c>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B12">
         <v>9</v>
       </c>
@@ -8461,7 +8868,7 @@
         <v>48.754109638160585</v>
       </c>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B13">
         <v>10</v>
       </c>
@@ -8470,7 +8877,7 @@
         <v>65.330506915135189</v>
       </c>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B14">
         <v>11</v>
       </c>
@@ -8479,7 +8886,7 @@
         <v>87.542879266281147</v>
       </c>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B15">
         <v>12</v>
       </c>
@@ -8492,7 +8899,7 @@
         <v>4090</v>
       </c>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B16">
         <v>13</v>
       </c>
@@ -8505,7 +8912,7 @@
         <v>5350</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B17">
         <v>14</v>
       </c>
@@ -8518,7 +8925,7 @@
         <v>7010</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B18">
         <v>15</v>
       </c>
@@ -8535,7 +8942,7 @@
         <v>14360</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B19">
         <v>16</v>
       </c>
@@ -8552,7 +8959,7 @@
         <v>18810</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B20">
         <v>17</v>
       </c>
@@ -8569,7 +8976,7 @@
         <v>24630</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B21">
         <v>18</v>
       </c>
@@ -8586,7 +8993,7 @@
         <v>32270</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B22">
         <v>19</v>
       </c>
@@ -8603,7 +9010,7 @@
         <v>42280</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B23">
         <v>20</v>
       </c>
@@ -8620,7 +9027,7 @@
         <v>55380</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B24">
         <v>21</v>
       </c>
@@ -8637,7 +9044,7 @@
         <v>72550</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B25">
         <v>22</v>
       </c>
@@ -8654,7 +9061,7 @@
         <v>95040</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B26">
         <v>23</v>
       </c>
@@ -8671,7 +9078,7 @@
         <v>124500</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B27">
         <v>24</v>
       </c>
@@ -8688,7 +9095,7 @@
         <v>163100</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B28">
         <v>25</v>
       </c>
@@ -8714,12 +9121,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B3:H15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B3" s="12" t="s">
         <v>69</v>
       </c>
@@ -8742,7 +9149,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>75</v>
       </c>
@@ -8767,7 +9174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>76</v>
       </c>
@@ -8792,7 +9199,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>77</v>
       </c>
@@ -8817,7 +9224,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>78</v>
       </c>
@@ -8842,7 +9249,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>79</v>
       </c>
@@ -8867,7 +9274,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>80</v>
       </c>
@@ -8892,7 +9299,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>81</v>
       </c>
@@ -8917,7 +9324,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>82</v>
       </c>
@@ -8942,7 +9349,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>83</v>
       </c>
@@ -8967,7 +9374,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>84</v>
       </c>
@@ -8992,7 +9399,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>85</v>
       </c>
@@ -9017,7 +9424,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>86</v>
       </c>
@@ -9051,12 +9458,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:E15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="2" max="2" width="10.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B2" s="11" t="s">
         <v>13</v>
       </c>
@@ -9064,7 +9471,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B3" s="11" t="s">
         <v>7</v>
       </c>
@@ -9072,7 +9479,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B4" s="11" t="s">
         <v>6</v>
       </c>
@@ -9080,7 +9487,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
         <v>15</v>
       </c>
@@ -9088,7 +9495,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B6" s="11" t="s">
         <v>16</v>
       </c>
@@ -9096,7 +9503,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B9" s="8" t="s">
         <v>11</v>
       </c>
@@ -9110,7 +9517,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B10">
         <v>1</v>
       </c>
@@ -9127,7 +9534,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B11">
         <v>2</v>
       </c>
@@ -9144,7 +9551,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B12">
         <v>3</v>
       </c>
@@ -9161,7 +9568,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B13">
         <v>4</v>
       </c>
@@ -9178,7 +9585,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B14">
         <v>5</v>
       </c>
@@ -9195,7 +9602,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B15">
         <v>6</v>
       </c>
@@ -9221,9 +9628,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:F28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B2" s="2" t="s">
         <v>51</v>
       </c>
@@ -9231,7 +9638,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B3" s="3">
         <v>1</v>
       </c>
@@ -9246,7 +9653,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B4" s="3">
         <v>2</v>
       </c>
@@ -9261,7 +9668,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B5" s="3">
         <v>3</v>
       </c>
@@ -9276,7 +9683,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B6" s="3">
         <v>4</v>
       </c>
@@ -9285,7 +9692,7 @@
         <v>13.2</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B7" s="3">
         <v>5</v>
       </c>
@@ -9294,7 +9701,7 @@
         <v>16.062305898749052</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B8" s="3">
         <v>6</v>
       </c>
@@ -9303,7 +9710,7 @@
         <v>19.227244611029164</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B9" s="3">
         <v>7</v>
       </c>
@@ -9312,7 +9719,7 @@
         <v>22.668233259706916</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B10" s="3">
         <v>8</v>
       </c>
@@ -9321,7 +9728,7 @@
         <v>26.364675298172557</v>
       </c>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B11" s="3">
         <v>9</v>
       </c>
@@ -9330,7 +9737,7 @@
         <v>30.3</v>
       </c>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B12" s="3">
         <v>10</v>
       </c>
@@ -9339,7 +9746,7 @@
         <v>34.460498941515425</v>
       </c>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B13" s="3">
         <v>11</v>
       </c>
@@ -9348,7 +9755,7 @@
         <v>38.834585424518465</v>
       </c>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B14" s="3">
         <v>12</v>
       </c>
@@ -9357,7 +9764,7 @@
         <v>43.412297443487766</v>
       </c>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B15" s="3">
         <v>13</v>
       </c>
@@ -9366,7 +9773,7 @@
         <v>48.184949922928681</v>
       </c>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B16" s="3">
         <v>14</v>
       </c>
@@ -9375,7 +9782,7 @@
         <v>53.144883073351636</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B17" s="3">
         <v>15</v>
       </c>
@@ -9384,7 +9791,7 @@
         <v>58.285275173800116</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B18" s="3">
         <v>16</v>
       </c>
@@ -9393,7 +9800,7 @@
         <v>63.59999999999998</v>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B19" s="3">
         <v>17</v>
       </c>
@@ -9402,7 +9809,7 @@
         <v>69.083516071950243</v>
       </c>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B20" s="3">
         <v>18</v>
       </c>
@@ -9411,7 +9818,7 @@
         <v>74.730779131332369</v>
       </c>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B21" s="3">
         <v>19</v>
       </c>
@@ -9420,7 +9827,7 @@
         <v>80.537171934545498</v>
       </c>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B22" s="3">
         <v>20</v>
       </c>
@@ -9429,7 +9836,7 @@
         <v>86.498447189992433</v>
       </c>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B23" s="3">
         <v>22</v>
       </c>
@@ -9438,7 +9845,7 @@
         <v>98.870232044503936</v>
       </c>
     </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B24" s="3">
         <v>24</v>
       </c>
@@ -9447,7 +9854,7 @@
         <v>111.81795688823334</v>
       </c>
     </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B25" s="3">
         <v>26</v>
       </c>
@@ -9456,7 +9863,7 @@
         <v>125.31705661807122</v>
       </c>
     </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B26" s="3">
         <v>28</v>
       </c>
@@ -9465,7 +9872,7 @@
         <v>139.3458660776553</v>
       </c>
     </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B27" s="3">
         <v>30</v>
       </c>
@@ -9474,7 +9881,7 @@
         <v>153.88509052639483</v>
       </c>
     </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B28" s="6"/>
       <c r="C28" s="29"/>
     </row>
@@ -9486,16 +9893,16 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:H27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
     </row>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B2" s="18" t="s">
         <v>54</v>
       </c>
@@ -9512,7 +9919,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B3" s="3">
         <v>0</v>
       </c>
@@ -9534,7 +9941,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B4" s="3">
         <v>1</v>
       </c>
@@ -9556,7 +9963,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B5" s="3">
         <v>2</v>
       </c>
@@ -9578,7 +9985,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B6" s="3">
         <v>4</v>
       </c>
@@ -9591,7 +9998,7 @@
         <v>90.144892671268622</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B7" s="3">
         <v>6</v>
       </c>
@@ -9604,7 +10011,7 @@
         <v>86.118675990610768</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B8" s="3">
         <v>8</v>
       </c>
@@ -9617,7 +10024,7 @@
         <v>82.3980943939046</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B9" s="3">
         <v>10</v>
       </c>
@@ -9630,7 +10037,7 @@
         <v>78.925220537571477</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B10" s="3">
         <v>15</v>
       </c>
@@ -9643,7 +10050,7 @@
         <v>71.113160110456874</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B11" s="3">
         <v>20</v>
       </c>
@@ -9656,7 +10063,7 @@
         <v>64.29806574927926</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B12" s="3">
         <v>25</v>
       </c>
@@ -9669,7 +10076,7 @@
         <v>58.282485186967683</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B13" s="3">
         <v>30</v>
       </c>
@@ -9682,7 +10089,7 @@
         <v>52.933290315596146</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B14" s="3">
         <v>35</v>
       </c>
@@ -9695,7 +10102,7 @@
         <v>48.151978235305769</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B15" s="3">
         <v>40</v>
       </c>
@@ -9708,7 +10115,7 @@
         <v>43.861617315434934</v>
       </c>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B16" s="3">
         <v>45</v>
       </c>
@@ -9721,7 +10128,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B17" s="3">
         <v>50</v>
       </c>
@@ -9734,7 +10141,7 @@
         <v>36.51560942092317</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B18" s="3">
         <v>60</v>
       </c>
@@ -9747,7 +10154,7 @@
         <v>30.511241564292174</v>
       </c>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B19" s="3">
         <v>70</v>
       </c>
@@ -9760,7 +10167,7 @@
         <v>25.570371161108223</v>
       </c>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B20" s="3">
         <v>80</v>
       </c>
@@ -9773,7 +10180,7 @@
         <v>21.48356373280761</v>
       </c>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B21" s="3">
         <v>90</v>
       </c>
@@ -9786,7 +10193,7 @@
         <v>18.089130275866257</v>
       </c>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B22" s="3">
         <v>100</v>
       </c>
@@ -9799,7 +10206,7 @@
         <v>15.260055429207236</v>
       </c>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B23" s="3">
         <v>120</v>
       </c>
@@ -9812,7 +10219,7 @@
         <v>10.913602200790223</v>
       </c>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B24" s="3">
         <v>140</v>
       </c>
@@ -9825,7 +10232,7 @@
         <v>7.8487089083892334</v>
       </c>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B25" s="3">
         <v>160</v>
       </c>
@@ -9838,7 +10245,7 @@
         <v>5.6710872889019068</v>
       </c>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B26" s="3">
         <v>180</v>
       </c>
@@ -9851,7 +10258,7 @@
         <v>4.1142663640113337</v>
       </c>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B27" s="3">
         <v>200</v>
       </c>
@@ -9874,23 +10281,23 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J50"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="4" width="0" hidden="1" customWidth="1"/>
-    <col min="8" max="9" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="8" max="9" width="9.1796875" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B5" s="12" t="s">
         <v>5</v>
       </c>
@@ -9908,7 +10315,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B6">
         <v>0</v>
       </c>
@@ -9940,7 +10347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B7">
         <v>200</v>
       </c>
@@ -9973,7 +10380,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B8">
         <v>400</v>
       </c>
@@ -10006,7 +10413,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B9">
         <v>600</v>
       </c>
@@ -10039,7 +10446,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B10">
         <v>800</v>
       </c>
@@ -10072,7 +10479,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B11">
         <v>1000</v>
       </c>
@@ -10105,7 +10512,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B12">
         <v>1500</v>
       </c>
@@ -10138,7 +10545,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B13">
         <v>2000</v>
       </c>
@@ -10171,7 +10578,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B14">
         <v>2500</v>
       </c>
@@ -10204,7 +10611,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B15">
         <v>3000</v>
       </c>
@@ -10237,7 +10644,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B16">
         <v>3500</v>
       </c>
@@ -10270,7 +10677,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B17">
         <v>4000</v>
       </c>
@@ -10303,7 +10710,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B18">
         <v>4500</v>
       </c>
@@ -10336,7 +10743,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B19">
         <v>5000</v>
       </c>
@@ -10369,7 +10776,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B20">
         <v>6000</v>
       </c>
@@ -10402,7 +10809,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B21">
         <v>7000</v>
       </c>
@@ -10435,7 +10842,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B22">
         <v>8000</v>
       </c>
@@ -10468,7 +10875,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B23">
         <v>9000</v>
       </c>
@@ -10501,7 +10908,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B24">
         <v>10000</v>
       </c>
@@ -10534,7 +10941,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B25">
         <v>11000</v>
       </c>
@@ -10567,7 +10974,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="26" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B26">
         <v>12000</v>
       </c>
@@ -10600,7 +11007,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="27" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B27">
         <v>13000</v>
       </c>
@@ -10633,7 +11040,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B28">
         <v>14000</v>
       </c>
@@ -10666,7 +11073,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B29">
         <v>15000</v>
       </c>
@@ -10699,7 +11106,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="30" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B30">
         <v>16000</v>
       </c>
@@ -10732,7 +11139,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="31" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B31">
         <v>17000</v>
       </c>
@@ -10765,7 +11172,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="32" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B32">
         <v>18000</v>
       </c>
@@ -10798,7 +11205,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B33">
         <v>19000</v>
       </c>
@@ -10831,7 +11238,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B34">
         <v>20000</v>
       </c>
@@ -10864,7 +11271,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B35">
         <v>21000</v>
       </c>
@@ -10897,7 +11304,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B36">
         <v>22000</v>
       </c>
@@ -10930,7 +11337,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B37">
         <v>23000</v>
       </c>
@@ -10963,7 +11370,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B38">
         <v>24000</v>
       </c>
@@ -10996,7 +11403,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B39">
         <v>25000</v>
       </c>
@@ -11029,7 +11436,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B40">
         <v>26000</v>
       </c>
@@ -11046,7 +11453,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="41" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B41">
         <v>27000</v>
       </c>
@@ -11063,7 +11470,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B42">
         <v>28000</v>
       </c>
@@ -11080,7 +11487,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B43">
         <v>29000</v>
       </c>
@@ -11097,7 +11504,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B44">
         <v>30000</v>
       </c>
@@ -11114,7 +11521,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B45">
         <v>31000</v>
       </c>
@@ -11131,7 +11538,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B46">
         <v>32000</v>
       </c>
@@ -11148,7 +11555,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B47">
         <v>33000</v>
       </c>
@@ -11165,7 +11572,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="48" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B48">
         <v>34000</v>
       </c>
@@ -11182,7 +11589,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B49">
         <v>35000</v>
       </c>
@@ -11199,7 +11606,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B50">
         <v>40000</v>
       </c>
@@ -11225,9 +11632,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:F22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
@@ -11235,7 +11642,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B3" s="3">
         <v>1</v>
       </c>
@@ -11250,7 +11657,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B4" s="3">
         <v>2</v>
       </c>
@@ -11265,7 +11672,7 @@
         <v>1.18</v>
       </c>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B5" s="3">
         <v>3</v>
       </c>
@@ -11280,7 +11687,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B6" s="3">
         <v>4</v>
       </c>
@@ -11289,7 +11696,7 @@
         <v>79.024488653385092</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B7" s="3">
         <v>5</v>
       </c>
@@ -11298,7 +11705,7 @@
         <v>133.06361577453981</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B8" s="3">
         <v>6</v>
       </c>
@@ -11307,7 +11714,7 @@
         <v>215.09394238321934</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B9" s="3">
         <v>7</v>
       </c>
@@ -11316,7 +11723,7 @@
         <v>338.03571078115363</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B10" s="3">
         <v>8</v>
       </c>
@@ -11325,7 +11732,7 @@
         <v>520.40581724408241</v>
       </c>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B11" s="3">
         <v>9</v>
       </c>
@@ -11334,7 +11741,7 @@
         <v>788.64631462151328</v>
       </c>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B12" s="3">
         <v>10</v>
       </c>
@@ -11343,7 +11750,7 @@
         <v>1180.3950561996239</v>
       </c>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B13" s="3">
         <v>11</v>
       </c>
@@ -11352,7 +11759,7 @@
         <v>1749.0719708434926</v>
       </c>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B14" s="3">
         <v>12</v>
       </c>
@@ -11361,7 +11768,7 @@
         <v>2570.300224997538</v>
       </c>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B15" s="3">
         <v>13</v>
       </c>
@@ -11370,7 +11777,7 @@
         <v>3750.8834844326066</v>
       </c>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B16" s="3">
         <v>14</v>
       </c>
@@ -11379,7 +11786,7 @@
         <v>5441.3400839676069</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B17" s="3">
         <v>15</v>
       </c>
@@ -11388,7 +11795,7 @@
         <v>7853.3817110156533</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B18" s="3">
         <v>16</v>
       </c>
@@ -11397,7 +11804,7 @@
         <v>11284.258942561721</v>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B19" s="3">
         <v>17</v>
       </c>
@@ -11406,7 +11813,7 @@
         <v>16150.634740535708</v>
       </c>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B20" s="3">
         <v>18</v>
       </c>
@@ -11415,7 +11822,7 @@
         <v>23035.667020966474</v>
       </c>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B21" s="3">
         <v>19</v>
       </c>
@@ -11424,7 +11831,7 @@
         <v>32754.388900956412</v>
       </c>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B22" s="3">
         <v>20</v>
       </c>

</xml_diff>